<commit_message>
Update NSE 200 DMA and fundamentals
</commit_message>
<xml_diff>
--- a/output/NSE_200DMA_Recovery_Scanner.xlsx
+++ b/output/NSE_200DMA_Recovery_Scanner.xlsx
@@ -644,7 +644,7 @@
         <v>81.13</v>
       </c>
       <c r="S2" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="T2" t="n">
         <v>452271374336</v>
@@ -742,7 +742,7 @@
         <v>17.08</v>
       </c>
       <c r="S3" t="n">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="T3" t="n">
         <v>114452561920</v>
@@ -831,51 +831,45 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>29.091524</v>
+        <v>28.993242</v>
       </c>
       <c r="Q4" t="n">
         <v>7.079106</v>
       </c>
       <c r="R4" t="n">
-        <v>5.9</v>
+        <v>5.92</v>
       </c>
       <c r="S4" t="n">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="T4" t="n">
         <v>1008188391424</v>
       </c>
-      <c r="U4" t="n">
-        <v>21.639</v>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="n">
-        <v>19.485001</v>
+        <v>19.645001</v>
       </c>
       <c r="X4" t="n">
-        <v>6.158</v>
+        <v>6.021</v>
       </c>
       <c r="Y4" t="n">
         <v>344.737</v>
       </c>
-      <c r="Z4" t="n">
-        <v>1.321</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>0.626</v>
-      </c>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="n">
-        <v>17.4</v>
+        <v>11.6</v>
       </c>
       <c r="AD4" t="n">
-        <v>24.5</v>
+        <v>1</v>
       </c>
       <c r="AE4" t="n">
-        <v>24.5</v>
+        <v>1</v>
       </c>
       <c r="AF4" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5">
@@ -1029,13 +1023,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>122.41681</v>
+        <v>98.03646000000001</v>
       </c>
       <c r="Q6" t="n">
         <v>12.074311</v>
       </c>
       <c r="R6" t="n">
-        <v>11.42</v>
+        <v>14.26</v>
       </c>
       <c r="S6" t="n">
         <v>37</v>
@@ -1142,7 +1136,7 @@
         <v>36.48</v>
       </c>
       <c r="S7" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="T7" t="n">
         <v>810549968896</v>
@@ -1335,13 +1329,13 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>58.438168</v>
+        <v>58.479492</v>
       </c>
       <c r="Q9" t="n">
         <v>9.402361000000001</v>
       </c>
       <c r="R9" t="n">
-        <v>14.15</v>
+        <v>14.14</v>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="n">
@@ -1529,13 +1523,13 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>38.17379</v>
+        <v>37.4601</v>
       </c>
       <c r="Q11" t="n">
         <v>5.515607</v>
       </c>
       <c r="R11" t="n">
-        <v>21.52</v>
+        <v>21.93</v>
       </c>
       <c r="S11" t="n">
         <v>72</v>
@@ -1734,7 +1728,7 @@
         <v>28.04</v>
       </c>
       <c r="S13" t="n">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="T13" t="n">
         <v>423900053504</v>
@@ -1823,16 +1817,16 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>9.728465</v>
+        <v>9.516741</v>
       </c>
       <c r="Q14" t="n">
         <v>2.097534</v>
       </c>
       <c r="R14" t="n">
-        <v>17.53</v>
+        <v>17.92</v>
       </c>
       <c r="S14" t="n">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="T14" t="n">
         <v>298888200192</v>
@@ -1917,13 +1911,13 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>16.460342</v>
+        <v>16.472553</v>
       </c>
       <c r="Q15" t="n">
         <v>1.6806881</v>
       </c>
       <c r="R15" t="n">
-        <v>26.98</v>
+        <v>26.96</v>
       </c>
       <c r="S15" t="n">
         <v>248</v>
@@ -2322,7 +2316,7 @@
         <v>108.37</v>
       </c>
       <c r="S19" t="n">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T19" t="n">
         <v>1338745946112</v>
@@ -2411,13 +2405,13 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>18.755718</v>
+        <v>18.760487</v>
       </c>
       <c r="Q20" t="n">
         <v>13.507057</v>
       </c>
       <c r="R20" t="n">
-        <v>39.34</v>
+        <v>39.33</v>
       </c>
       <c r="S20" t="n">
         <v>54</v>
@@ -2606,47 +2600,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; recovery &gt;=5%; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P22" t="n">
-        <v>5.337037</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>0.7214199</v>
-      </c>
-      <c r="R22" t="n">
-        <v>27</v>
-      </c>
-      <c r="S22" t="n">
-        <v>323</v>
-      </c>
-      <c r="T22" t="n">
-        <v>656039411712</v>
-      </c>
-      <c r="U22" t="n">
-        <v>13.697</v>
-      </c>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr"/>
-      <c r="W22" t="n">
-        <v>48.535</v>
-      </c>
-      <c r="X22" t="n">
-        <v>34.992</v>
-      </c>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
       <c r="AB22" t="inlineStr"/>
-      <c r="AC22" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="AD22" t="n">
-        <v>80.30000000000001</v>
-      </c>
-      <c r="AE22" t="n">
-        <v>80.30000000000001</v>
-      </c>
-      <c r="AF22" t="n">
-        <v>84</v>
-      </c>
+      <c r="AC22" t="inlineStr"/>
+      <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2704,47 +2674,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; recovery &gt;=5%; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P23" t="n">
-        <v>48.788597</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>12.517901</v>
-      </c>
-      <c r="R23" t="n">
-        <v>8.42</v>
-      </c>
-      <c r="S23" t="n">
-        <v>62</v>
-      </c>
-      <c r="T23" t="n">
-        <v>3002857160704</v>
-      </c>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr"/>
-      <c r="W23" t="n">
-        <v>22.135</v>
-      </c>
-      <c r="X23" t="n">
-        <v>21.403</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>0.273</v>
-      </c>
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr"/>
       <c r="AA23" t="inlineStr"/>
       <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="n">
-        <v>24.9</v>
-      </c>
-      <c r="AD23" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="AE23" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="AF23" t="n">
-        <v>76</v>
-      </c>
+      <c r="AC23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2802,45 +2748,23 @@
           <t>at/above 200DMA; moving toward 200DMA; above breakdown low; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P24" t="n">
-        <v>160.23636</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>4.3186584</v>
-      </c>
-      <c r="R24" t="n">
-        <v>2.75</v>
-      </c>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
-      <c r="T24" t="n">
-        <v>168591523840</v>
-      </c>
+      <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr"/>
-      <c r="W24" t="n">
-        <v>-11.457</v>
-      </c>
-      <c r="X24" t="n">
-        <v>4.961</v>
-      </c>
-      <c r="Y24" t="n">
-        <v>9.928000000000001</v>
-      </c>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="inlineStr"/>
       <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="n">
-        <v>-23.1</v>
-      </c>
-      <c r="AD24" t="n">
-        <v>-96.8</v>
-      </c>
-      <c r="AE24" t="n">
-        <v>-96.8</v>
-      </c>
-      <c r="AF24" t="n">
-        <v>8</v>
-      </c>
+      <c r="AC24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2898,47 +2822,23 @@
           <t>at/above 200DMA; moving toward 200DMA; recovery &gt;=5%; above 50DMA</t>
         </is>
       </c>
-      <c r="P25" t="n">
-        <v>25.438437</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>3.9687612</v>
-      </c>
-      <c r="R25" t="n">
-        <v>8.69</v>
-      </c>
-      <c r="S25" t="n">
-        <v>249</v>
-      </c>
-      <c r="T25" t="n">
-        <v>106242269184</v>
-      </c>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr"/>
-      <c r="W25" t="n">
-        <v>18.431</v>
-      </c>
-      <c r="X25" t="n">
-        <v>16.983</v>
-      </c>
-      <c r="Y25" t="n">
-        <v>0.236</v>
-      </c>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="inlineStr"/>
       <c r="AB25" t="inlineStr"/>
-      <c r="AC25" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="AD25" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="AE25" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="AF25" t="n">
-        <v>64</v>
-      </c>
+      <c r="AC25" t="inlineStr"/>
+      <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2996,47 +2896,23 @@
           <t>at/above 200DMA; recovery &gt;=5%; above 50DMA; volume &gt;=1.2x; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P26" t="n">
-        <v>54.039127</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>6.0853057</v>
-      </c>
-      <c r="R26" t="n">
-        <v>17.38</v>
-      </c>
-      <c r="S26" t="n">
-        <v>21</v>
-      </c>
-      <c r="T26" t="n">
-        <v>239427633152</v>
-      </c>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr"/>
-      <c r="W26" t="n">
-        <v>17.254</v>
-      </c>
-      <c r="X26" t="n">
-        <v>8.457000000000001</v>
-      </c>
-      <c r="Y26" t="n">
-        <v>55.868</v>
-      </c>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
       <c r="Z26" t="inlineStr"/>
       <c r="AA26" t="inlineStr"/>
       <c r="AB26" t="inlineStr"/>
-      <c r="AC26" t="n">
-        <v>15</v>
-      </c>
-      <c r="AD26" t="n">
-        <v>153.2</v>
-      </c>
-      <c r="AE26" t="n">
-        <v>153.2</v>
-      </c>
-      <c r="AF26" t="n">
-        <v>42</v>
-      </c>
+      <c r="AC26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -3095,44 +2971,22 @@
         </is>
       </c>
       <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="n">
-        <v>4.1930685</v>
-      </c>
-      <c r="R27" t="n">
-        <v>-31.78</v>
-      </c>
-      <c r="S27" t="n">
-        <v>18</v>
-      </c>
-      <c r="T27" t="n">
-        <v>155129659392</v>
-      </c>
-      <c r="U27" t="n">
-        <v>-8.911</v>
-      </c>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
-      <c r="W27" t="n">
-        <v>-186.002</v>
-      </c>
-      <c r="X27" t="n">
-        <v>-24.914</v>
-      </c>
-      <c r="Y27" t="n">
-        <v>152.371</v>
-      </c>
-      <c r="Z27" t="n">
-        <v>1.437</v>
-      </c>
-      <c r="AA27" t="n">
-        <v>0.252</v>
-      </c>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
       <c r="AB27" t="inlineStr"/>
       <c r="AC27" t="inlineStr"/>
       <c r="AD27" t="inlineStr"/>
       <c r="AE27" t="inlineStr"/>
-      <c r="AF27" t="n">
-        <v>12</v>
-      </c>
+      <c r="AF27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -3190,45 +3044,23 @@
           <t>at/above 200DMA; moving toward 200DMA; recovery &gt;=5%; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P28" t="n">
-        <v>86.733604</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>10.799423</v>
-      </c>
-      <c r="R28" t="n">
-        <v>46.81</v>
-      </c>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
-      <c r="T28" t="n">
-        <v>2648118657024</v>
-      </c>
+      <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr"/>
-      <c r="W28" t="n">
-        <v>6.447</v>
-      </c>
-      <c r="X28" t="n">
-        <v>4.2919997</v>
-      </c>
-      <c r="Y28" t="n">
-        <v>9.913</v>
-      </c>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
       <c r="AA28" t="inlineStr"/>
       <c r="AB28" t="inlineStr"/>
-      <c r="AC28" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="AD28" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="AE28" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="AF28" t="n">
-        <v>36</v>
-      </c>
+      <c r="AC28" t="inlineStr"/>
+      <c r="AD28" t="inlineStr"/>
+      <c r="AE28" t="inlineStr"/>
+      <c r="AF28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -3286,53 +3118,23 @@
           <t>at/above 200DMA; moving toward 200DMA; recovery &gt;=5%; volume &gt;=1.2x</t>
         </is>
       </c>
-      <c r="P29" t="n">
-        <v>50.43283</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>10.30154</v>
-      </c>
-      <c r="R29" t="n">
-        <v>80.17</v>
-      </c>
-      <c r="S29" t="n">
-        <v>85</v>
-      </c>
-      <c r="T29" t="n">
-        <v>631966990336</v>
-      </c>
-      <c r="U29" t="n">
-        <v>21.645</v>
-      </c>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr"/>
-      <c r="W29" t="n">
-        <v>14.774999</v>
-      </c>
-      <c r="X29" t="n">
-        <v>11.9320005</v>
-      </c>
-      <c r="Y29" t="n">
-        <v>0.783</v>
-      </c>
-      <c r="Z29" t="n">
-        <v>2.487</v>
-      </c>
-      <c r="AA29" t="n">
-        <v>1.423</v>
-      </c>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
       <c r="AB29" t="inlineStr"/>
-      <c r="AC29" t="n">
-        <v>17.3</v>
-      </c>
-      <c r="AD29" t="n">
-        <v>13</v>
-      </c>
-      <c r="AE29" t="n">
-        <v>13</v>
-      </c>
-      <c r="AF29" t="n">
-        <v>69</v>
-      </c>
+      <c r="AC29" t="inlineStr"/>
+      <c r="AD29" t="inlineStr"/>
+      <c r="AE29" t="inlineStr"/>
+      <c r="AF29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -3390,53 +3192,23 @@
           <t>at/above 200DMA; recovery &gt;=10%; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P30" t="n">
-        <v>29.951899</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>28.286232</v>
-      </c>
-      <c r="R30" t="n">
-        <v>19.75</v>
-      </c>
-      <c r="S30" t="n">
-        <v>34</v>
-      </c>
-      <c r="T30" t="n">
-        <v>192941342720</v>
-      </c>
-      <c r="U30" t="n">
-        <v>10.786</v>
-      </c>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr"/>
-      <c r="W30" t="n">
-        <v>20.204</v>
-      </c>
-      <c r="X30" t="n">
-        <v>11.311</v>
-      </c>
-      <c r="Y30" t="n">
-        <v>84.316</v>
-      </c>
-      <c r="Z30" t="n">
-        <v>1.241</v>
-      </c>
-      <c r="AA30" t="n">
-        <v>0.26</v>
-      </c>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
       <c r="AB30" t="inlineStr"/>
-      <c r="AC30" t="n">
-        <v>-0.2</v>
-      </c>
-      <c r="AD30" t="n">
-        <v>-42.3</v>
-      </c>
-      <c r="AE30" t="n">
-        <v>-42.3</v>
-      </c>
-      <c r="AF30" t="n">
-        <v>34</v>
-      </c>
+      <c r="AC30" t="inlineStr"/>
+      <c r="AD30" t="inlineStr"/>
+      <c r="AE30" t="inlineStr"/>
+      <c r="AF30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -3444,7 +3216,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>M%26M</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3494,47 +3266,23 @@
           <t>at/above 200DMA; recovery &gt;=10%; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P31" t="n">
-        <v>20.877535</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>4.115483</v>
-      </c>
-      <c r="R31" t="n">
-        <v>164.21</v>
-      </c>
-      <c r="S31" t="n">
-        <v>0.9599999499999999</v>
-      </c>
-      <c r="T31" t="n">
-        <v>4116573323264</v>
-      </c>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr"/>
-      <c r="W31" t="n">
-        <v>17.031</v>
-      </c>
-      <c r="X31" t="n">
-        <v>8.609</v>
-      </c>
-      <c r="Y31" t="n">
-        <v>125.278</v>
-      </c>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr"/>
       <c r="AA31" t="inlineStr"/>
       <c r="AB31" t="inlineStr"/>
-      <c r="AC31" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="AD31" t="n">
-        <v>33.4</v>
-      </c>
-      <c r="AE31" t="n">
-        <v>33.4</v>
-      </c>
-      <c r="AF31" t="n">
-        <v>62</v>
-      </c>
+      <c r="AC31" t="inlineStr"/>
+      <c r="AD31" t="inlineStr"/>
+      <c r="AE31" t="inlineStr"/>
+      <c r="AF31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -3592,47 +3340,23 @@
           <t>at/above 200DMA; recovery &gt;=10%; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P32" t="n">
-        <v>6.1426344</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>0.86730266</v>
-      </c>
-      <c r="R32" t="n">
-        <v>19.21</v>
-      </c>
-      <c r="S32" t="n">
-        <v>255</v>
-      </c>
-      <c r="T32" t="n">
-        <v>1356167249920</v>
-      </c>
-      <c r="U32" t="n">
-        <v>14.965999</v>
-      </c>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr"/>
-      <c r="W32" t="n">
-        <v>29.405</v>
-      </c>
-      <c r="X32" t="n">
-        <v>38.147</v>
-      </c>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
       <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr"/>
       <c r="AA32" t="inlineStr"/>
       <c r="AB32" t="inlineStr"/>
-      <c r="AC32" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="AD32" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="AE32" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="AF32" t="n">
-        <v>72</v>
-      </c>
+      <c r="AC32" t="inlineStr"/>
+      <c r="AD32" t="inlineStr"/>
+      <c r="AE32" t="inlineStr"/>
+      <c r="AF32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -3690,17 +3414,11 @@
           <t>at/above 200DMA; recovery &gt;=10%; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P33" t="n">
-        <v>7.347592</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>5.883686</v>
-      </c>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
-      <c r="T33" t="n">
-        <v>144244375552</v>
-      </c>
+      <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr"/>
       <c r="W33" t="inlineStr"/>
@@ -3712,9 +3430,7 @@
       <c r="AC33" t="inlineStr"/>
       <c r="AD33" t="inlineStr"/>
       <c r="AE33" t="inlineStr"/>
-      <c r="AF33" t="n">
-        <v>100</v>
-      </c>
+      <c r="AF33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -3772,53 +3488,23 @@
           <t>at/above 200DMA; recovery &gt;=10%; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P34" t="n">
-        <v>25.444912</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>4.2841005</v>
-      </c>
-      <c r="R34" t="n">
-        <v>100.02</v>
-      </c>
-      <c r="S34" t="n">
-        <v>244</v>
-      </c>
-      <c r="T34" t="n">
-        <v>485629394944</v>
-      </c>
-      <c r="U34" t="n">
-        <v>17.743999</v>
-      </c>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr"/>
-      <c r="W34" t="n">
-        <v>14.783</v>
-      </c>
-      <c r="X34" t="n">
-        <v>11.5559995</v>
-      </c>
-      <c r="Y34" t="n">
-        <v>24.675</v>
-      </c>
-      <c r="Z34" t="n">
-        <v>1.459</v>
-      </c>
-      <c r="AA34" t="n">
-        <v>1.265</v>
-      </c>
+      <c r="W34" t="inlineStr"/>
+      <c r="X34" t="inlineStr"/>
+      <c r="Y34" t="inlineStr"/>
+      <c r="Z34" t="inlineStr"/>
+      <c r="AA34" t="inlineStr"/>
       <c r="AB34" t="inlineStr"/>
-      <c r="AC34" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="AD34" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="AE34" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="AF34" t="n">
-        <v>59</v>
-      </c>
+      <c r="AC34" t="inlineStr"/>
+      <c r="AD34" t="inlineStr"/>
+      <c r="AE34" t="inlineStr"/>
+      <c r="AF34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -3876,53 +3562,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; above breakdown low; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P35" t="n">
-        <v>26.16391</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>5.177395</v>
-      </c>
-      <c r="R35" t="n">
-        <v>21.78</v>
-      </c>
-      <c r="S35" t="n">
-        <v>248</v>
-      </c>
-      <c r="T35" t="n">
-        <v>347489959936</v>
-      </c>
-      <c r="U35" t="n">
-        <v>21.473</v>
-      </c>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr"/>
-      <c r="W35" t="n">
-        <v>13.739</v>
-      </c>
-      <c r="X35" t="n">
-        <v>9.318</v>
-      </c>
-      <c r="Y35" t="n">
-        <v>10.18</v>
-      </c>
-      <c r="Z35" t="n">
-        <v>1.432</v>
-      </c>
-      <c r="AA35" t="n">
-        <v>1.121</v>
-      </c>
+      <c r="W35" t="inlineStr"/>
+      <c r="X35" t="inlineStr"/>
+      <c r="Y35" t="inlineStr"/>
+      <c r="Z35" t="inlineStr"/>
+      <c r="AA35" t="inlineStr"/>
       <c r="AB35" t="inlineStr"/>
-      <c r="AC35" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="AD35" t="n">
-        <v>-12.5</v>
-      </c>
-      <c r="AE35" t="n">
-        <v>-12.5</v>
-      </c>
-      <c r="AF35" t="n">
-        <v>47</v>
-      </c>
+      <c r="AC35" t="inlineStr"/>
+      <c r="AD35" t="inlineStr"/>
+      <c r="AE35" t="inlineStr"/>
+      <c r="AF35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3980,47 +3636,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; above breakdown low; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P36" t="n">
-        <v>14.326874</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>10.491822</v>
-      </c>
-      <c r="R36" t="n">
-        <v>39.22</v>
-      </c>
-      <c r="S36" t="n">
-        <v>374</v>
-      </c>
-      <c r="T36" t="n">
-        <v>2374206750720</v>
-      </c>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr"/>
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr"/>
-      <c r="W36" t="n">
-        <v>54.70699999999999</v>
-      </c>
-      <c r="X36" t="n">
-        <v>38.068</v>
-      </c>
-      <c r="Y36" t="n">
-        <v>39.034</v>
-      </c>
+      <c r="W36" t="inlineStr"/>
+      <c r="X36" t="inlineStr"/>
+      <c r="Y36" t="inlineStr"/>
       <c r="Z36" t="inlineStr"/>
       <c r="AA36" t="inlineStr"/>
       <c r="AB36" t="inlineStr"/>
-      <c r="AC36" t="n">
-        <v>71.7</v>
-      </c>
-      <c r="AD36" t="n">
-        <v>144.6</v>
-      </c>
-      <c r="AE36" t="n">
-        <v>144.6</v>
-      </c>
-      <c r="AF36" t="n">
-        <v>80</v>
-      </c>
+      <c r="AC36" t="inlineStr"/>
+      <c r="AD36" t="inlineStr"/>
+      <c r="AE36" t="inlineStr"/>
+      <c r="AF36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -4078,53 +3710,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; above breakdown low; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P37" t="n">
-        <v>59.513058</v>
-      </c>
-      <c r="Q37" t="n">
-        <v>14.337361</v>
-      </c>
-      <c r="R37" t="n">
-        <v>22.59</v>
-      </c>
-      <c r="S37" t="n">
-        <v>95</v>
-      </c>
-      <c r="T37" t="n">
-        <v>280979603456</v>
-      </c>
-      <c r="U37" t="n">
-        <v>23.913</v>
-      </c>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr"/>
-      <c r="W37" t="n">
-        <v>38.09</v>
-      </c>
-      <c r="X37" t="n">
-        <v>36.923</v>
-      </c>
-      <c r="Y37" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="Z37" t="n">
-        <v>2.917</v>
-      </c>
-      <c r="AA37" t="n">
-        <v>2.464</v>
-      </c>
+      <c r="W37" t="inlineStr"/>
+      <c r="X37" t="inlineStr"/>
+      <c r="Y37" t="inlineStr"/>
+      <c r="Z37" t="inlineStr"/>
+      <c r="AA37" t="inlineStr"/>
       <c r="AB37" t="inlineStr"/>
-      <c r="AC37" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="AD37" t="n">
-        <v>-19.9</v>
-      </c>
-      <c r="AE37" t="n">
-        <v>-19.9</v>
-      </c>
-      <c r="AF37" t="n">
-        <v>63</v>
-      </c>
+      <c r="AC37" t="inlineStr"/>
+      <c r="AD37" t="inlineStr"/>
+      <c r="AE37" t="inlineStr"/>
+      <c r="AF37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -4182,53 +3784,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; above breakdown low; above 50DMA; volume &gt;=1.2x</t>
         </is>
       </c>
-      <c r="P38" t="n">
-        <v>35.626358</v>
-      </c>
-      <c r="Q38" t="n">
-        <v>12.044059</v>
-      </c>
-      <c r="R38" t="n">
-        <v>759.55</v>
-      </c>
-      <c r="S38" t="n">
-        <v>190</v>
-      </c>
-      <c r="T38" t="n">
-        <v>575006113792</v>
-      </c>
-      <c r="U38" t="n">
-        <v>34.460998</v>
-      </c>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr"/>
-      <c r="W38" t="n">
-        <v>27.021</v>
-      </c>
-      <c r="X38" t="n">
-        <v>22.399001</v>
-      </c>
-      <c r="Y38" t="n">
-        <v>3.602</v>
-      </c>
-      <c r="Z38" t="n">
-        <v>2.554</v>
-      </c>
-      <c r="AA38" t="n">
-        <v>1.878</v>
-      </c>
+      <c r="W38" t="inlineStr"/>
+      <c r="X38" t="inlineStr"/>
+      <c r="Y38" t="inlineStr"/>
+      <c r="Z38" t="inlineStr"/>
+      <c r="AA38" t="inlineStr"/>
       <c r="AB38" t="inlineStr"/>
-      <c r="AC38" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="AD38" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="AE38" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="AF38" t="n">
-        <v>60</v>
-      </c>
+      <c r="AC38" t="inlineStr"/>
+      <c r="AD38" t="inlineStr"/>
+      <c r="AE38" t="inlineStr"/>
+      <c r="AF38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -4286,45 +3858,23 @@
           <t>at/above 200DMA; moving toward 200DMA; above breakdown low; above 50DMA</t>
         </is>
       </c>
-      <c r="P39" t="n">
-        <v>31.160711</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>1.157679</v>
-      </c>
-      <c r="R39" t="n">
-        <v>10.64</v>
-      </c>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr"/>
-      <c r="T39" t="n">
-        <v>118415122432</v>
-      </c>
+      <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr"/>
       <c r="V39" t="inlineStr"/>
-      <c r="W39" t="n">
-        <v>10.953</v>
-      </c>
-      <c r="X39" t="n">
-        <v>3.329</v>
-      </c>
-      <c r="Y39" t="n">
-        <v>48.061</v>
-      </c>
+      <c r="W39" t="inlineStr"/>
+      <c r="X39" t="inlineStr"/>
+      <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr"/>
       <c r="AA39" t="inlineStr"/>
       <c r="AB39" t="inlineStr"/>
-      <c r="AC39" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="AD39" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="AE39" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="AF39" t="n">
-        <v>38</v>
-      </c>
+      <c r="AC39" t="inlineStr"/>
+      <c r="AD39" t="inlineStr"/>
+      <c r="AE39" t="inlineStr"/>
+      <c r="AF39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -4382,47 +3932,23 @@
           <t>at/above 200DMA; moving toward 200DMA; above breakdown low; above 50DMA</t>
         </is>
       </c>
-      <c r="P40" t="n">
-        <v>34.12324</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>4.882711</v>
-      </c>
-      <c r="R40" t="n">
-        <v>24.18</v>
-      </c>
-      <c r="S40" t="n">
-        <v>24</v>
-      </c>
-      <c r="T40" t="n">
-        <v>180692041728</v>
-      </c>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr"/>
       <c r="U40" t="inlineStr"/>
       <c r="V40" t="inlineStr"/>
-      <c r="W40" t="n">
-        <v>33.731</v>
-      </c>
-      <c r="X40" t="n">
-        <v>22.12</v>
-      </c>
-      <c r="Y40" t="n">
-        <v>64.041</v>
-      </c>
+      <c r="W40" t="inlineStr"/>
+      <c r="X40" t="inlineStr"/>
+      <c r="Y40" t="inlineStr"/>
       <c r="Z40" t="inlineStr"/>
       <c r="AA40" t="inlineStr"/>
       <c r="AB40" t="inlineStr"/>
-      <c r="AC40" t="n">
-        <v>-42.7</v>
-      </c>
-      <c r="AD40" t="n">
-        <v>-57.7</v>
-      </c>
-      <c r="AE40" t="n">
-        <v>-57.7</v>
-      </c>
-      <c r="AF40" t="n">
-        <v>28</v>
-      </c>
+      <c r="AC40" t="inlineStr"/>
+      <c r="AD40" t="inlineStr"/>
+      <c r="AE40" t="inlineStr"/>
+      <c r="AF40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -4480,45 +4006,23 @@
           <t>at/above 200DMA; moving toward 200DMA; recovery &gt;=10%</t>
         </is>
       </c>
-      <c r="P41" t="n">
-        <v>104.28282</v>
-      </c>
-      <c r="Q41" t="n">
-        <v>13.3846655</v>
-      </c>
-      <c r="R41" t="n">
-        <v>64.20999999999999</v>
-      </c>
-      <c r="S41" t="n">
-        <v>6</v>
-      </c>
-      <c r="T41" t="n">
-        <v>571063140352</v>
-      </c>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
       <c r="V41" t="inlineStr"/>
-      <c r="W41" t="n">
-        <v>20.444</v>
-      </c>
-      <c r="X41" t="n">
-        <v>20.587</v>
-      </c>
+      <c r="W41" t="inlineStr"/>
+      <c r="X41" t="inlineStr"/>
       <c r="Y41" t="inlineStr"/>
       <c r="Z41" t="inlineStr"/>
       <c r="AA41" t="inlineStr"/>
       <c r="AB41" t="inlineStr"/>
-      <c r="AC41" t="n">
-        <v>13.1</v>
-      </c>
-      <c r="AD41" t="n">
-        <v>676.4</v>
-      </c>
-      <c r="AE41" t="n">
-        <v>676.4</v>
-      </c>
-      <c r="AF41" t="n">
-        <v>68</v>
-      </c>
+      <c r="AC41" t="inlineStr"/>
+      <c r="AD41" t="inlineStr"/>
+      <c r="AE41" t="inlineStr"/>
+      <c r="AF41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -4576,47 +4080,23 @@
           <t>at/above 200DMA; moving toward 200DMA; recovery &gt;=10%</t>
         </is>
       </c>
-      <c r="P42" t="n">
-        <v>26.382</v>
-      </c>
-      <c r="Q42" t="n">
-        <v>4.2775254</v>
-      </c>
-      <c r="R42" t="n">
-        <v>10.89</v>
-      </c>
-      <c r="S42" t="n">
-        <v>173</v>
-      </c>
-      <c r="T42" t="n">
-        <v>262502383616</v>
-      </c>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr"/>
-      <c r="W42" t="n">
-        <v>24.655001</v>
-      </c>
-      <c r="X42" t="n">
-        <v>20.698</v>
-      </c>
-      <c r="Y42" t="n">
-        <v>129.314</v>
-      </c>
+      <c r="W42" t="inlineStr"/>
+      <c r="X42" t="inlineStr"/>
+      <c r="Y42" t="inlineStr"/>
       <c r="Z42" t="inlineStr"/>
       <c r="AA42" t="inlineStr"/>
       <c r="AB42" t="inlineStr"/>
-      <c r="AC42" t="n">
-        <v>23</v>
-      </c>
-      <c r="AD42" t="n">
-        <v>100</v>
-      </c>
-      <c r="AE42" t="n">
-        <v>100</v>
-      </c>
-      <c r="AF42" t="n">
-        <v>74</v>
-      </c>
+      <c r="AC42" t="inlineStr"/>
+      <c r="AD42" t="inlineStr"/>
+      <c r="AE42" t="inlineStr"/>
+      <c r="AF42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -4674,47 +4154,23 @@
           <t>at/above 200DMA; recovery &gt;=5%; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P43" t="n">
-        <v>16.582893</v>
-      </c>
-      <c r="Q43" t="n">
-        <v>2.5415702</v>
-      </c>
-      <c r="R43" t="n">
-        <v>32.03</v>
-      </c>
-      <c r="S43" t="n">
-        <v>38</v>
-      </c>
-      <c r="T43" t="n">
-        <v>187167326208</v>
-      </c>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr"/>
-      <c r="W43" t="n">
-        <v>35.115</v>
-      </c>
-      <c r="X43" t="n">
-        <v>19.941</v>
-      </c>
-      <c r="Y43" t="n">
-        <v>35.204</v>
-      </c>
+      <c r="W43" t="inlineStr"/>
+      <c r="X43" t="inlineStr"/>
+      <c r="Y43" t="inlineStr"/>
       <c r="Z43" t="inlineStr"/>
       <c r="AA43" t="inlineStr"/>
       <c r="AB43" t="inlineStr"/>
-      <c r="AC43" t="n">
-        <v>-1.5</v>
-      </c>
-      <c r="AD43" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="AE43" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="AF43" t="n">
-        <v>42</v>
-      </c>
+      <c r="AC43" t="inlineStr"/>
+      <c r="AD43" t="inlineStr"/>
+      <c r="AE43" t="inlineStr"/>
+      <c r="AF43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -4772,47 +4228,23 @@
           <t>at/above 200DMA; recovery &gt;=5%; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P44" t="n">
-        <v>33.782997</v>
-      </c>
-      <c r="Q44" t="n">
-        <v>5.1065493</v>
-      </c>
-      <c r="R44" t="n">
-        <v>120.09</v>
-      </c>
-      <c r="S44" t="n">
-        <v>93</v>
-      </c>
-      <c r="T44" t="n">
-        <v>5581888815104</v>
-      </c>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr"/>
-      <c r="W44" t="n">
-        <v>10.609999</v>
-      </c>
-      <c r="X44" t="n">
-        <v>5.588</v>
-      </c>
-      <c r="Y44" t="n">
-        <v>97.64</v>
-      </c>
+      <c r="W44" t="inlineStr"/>
+      <c r="X44" t="inlineStr"/>
+      <c r="Y44" t="inlineStr"/>
       <c r="Z44" t="inlineStr"/>
       <c r="AA44" t="inlineStr"/>
       <c r="AB44" t="inlineStr"/>
-      <c r="AC44" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="AD44" t="n">
-        <v>14</v>
-      </c>
-      <c r="AE44" t="n">
-        <v>14</v>
-      </c>
-      <c r="AF44" t="n">
-        <v>38</v>
-      </c>
+      <c r="AC44" t="inlineStr"/>
+      <c r="AD44" t="inlineStr"/>
+      <c r="AE44" t="inlineStr"/>
+      <c r="AF44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -4870,53 +4302,23 @@
           <t>at/above 200DMA; above breakdown low; above 50DMA; volume &gt;=1.2x; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P45" t="n">
-        <v>40.489838</v>
-      </c>
-      <c r="Q45" t="n">
-        <v>7.677307</v>
-      </c>
-      <c r="R45" t="n">
-        <v>49.2</v>
-      </c>
-      <c r="S45" t="n">
-        <v>124</v>
-      </c>
-      <c r="T45" t="n">
-        <v>12428031033344</v>
-      </c>
-      <c r="U45" t="n">
-        <v>20.151</v>
-      </c>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr"/>
+      <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr"/>
-      <c r="W45" t="n">
-        <v>32.573003</v>
-      </c>
-      <c r="X45" t="n">
-        <v>13.14</v>
-      </c>
-      <c r="Y45" t="n">
-        <v>100.415</v>
-      </c>
-      <c r="Z45" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="AA45" t="n">
-        <v>0.358</v>
-      </c>
+      <c r="W45" t="inlineStr"/>
+      <c r="X45" t="inlineStr"/>
+      <c r="Y45" t="inlineStr"/>
+      <c r="Z45" t="inlineStr"/>
+      <c r="AA45" t="inlineStr"/>
       <c r="AB45" t="inlineStr"/>
-      <c r="AC45" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="AD45" t="n">
-        <v>35.09999999999999</v>
-      </c>
-      <c r="AE45" t="n">
-        <v>35.09999999999999</v>
-      </c>
-      <c r="AF45" t="n">
-        <v>54</v>
-      </c>
+      <c r="AC45" t="inlineStr"/>
+      <c r="AD45" t="inlineStr"/>
+      <c r="AE45" t="inlineStr"/>
+      <c r="AF45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -4974,47 +4376,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; above breakdown low; volume &gt;=1.2x; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P46" t="n">
-        <v>31.679102</v>
-      </c>
-      <c r="Q46" t="n">
-        <v>3.0924454</v>
-      </c>
-      <c r="R46" t="n">
-        <v>12.06</v>
-      </c>
-      <c r="S46" t="n">
-        <v>65</v>
-      </c>
-      <c r="T46" t="n">
-        <v>1220779442176</v>
-      </c>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr"/>
-      <c r="W46" t="n">
-        <v>14.453</v>
-      </c>
-      <c r="X46" t="n">
-        <v>6.0890004</v>
-      </c>
-      <c r="Y46" t="n">
-        <v>168.051</v>
-      </c>
+      <c r="W46" t="inlineStr"/>
+      <c r="X46" t="inlineStr"/>
+      <c r="Y46" t="inlineStr"/>
       <c r="Z46" t="inlineStr"/>
       <c r="AA46" t="inlineStr"/>
       <c r="AB46" t="inlineStr"/>
-      <c r="AC46" t="n">
-        <v>5.600000000000001</v>
-      </c>
-      <c r="AD46" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="AE46" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="AF46" t="n">
-        <v>38</v>
-      </c>
+      <c r="AC46" t="inlineStr"/>
+      <c r="AD46" t="inlineStr"/>
+      <c r="AE46" t="inlineStr"/>
+      <c r="AF46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -5072,53 +4450,23 @@
           <t>at/above 200DMA; moving toward 200DMA; above breakdown low; volume &gt;=1.2x</t>
         </is>
       </c>
-      <c r="P47" t="n">
-        <v>54.102196</v>
-      </c>
-      <c r="Q47" t="n">
-        <v>27.279732</v>
-      </c>
-      <c r="R47" t="n">
-        <v>679.27</v>
-      </c>
-      <c r="S47" t="n">
-        <v>157</v>
-      </c>
-      <c r="T47" t="n">
-        <v>409904873472</v>
-      </c>
-      <c r="U47" t="n">
-        <v>52.5</v>
-      </c>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="inlineStr"/>
       <c r="V47" t="inlineStr"/>
-      <c r="W47" t="n">
-        <v>18.868999</v>
-      </c>
-      <c r="X47" t="n">
-        <v>14.558</v>
-      </c>
-      <c r="Y47" t="n">
-        <v>18.422</v>
-      </c>
-      <c r="Z47" t="n">
-        <v>1.725</v>
-      </c>
-      <c r="AA47" t="n">
-        <v>0.5669999999999999</v>
-      </c>
+      <c r="W47" t="inlineStr"/>
+      <c r="X47" t="inlineStr"/>
+      <c r="Y47" t="inlineStr"/>
+      <c r="Z47" t="inlineStr"/>
+      <c r="AA47" t="inlineStr"/>
       <c r="AB47" t="inlineStr"/>
-      <c r="AC47" t="n">
-        <v>14.1</v>
-      </c>
-      <c r="AD47" t="n">
-        <v>9</v>
-      </c>
-      <c r="AE47" t="n">
-        <v>9</v>
-      </c>
-      <c r="AF47" t="n">
-        <v>51</v>
-      </c>
+      <c r="AC47" t="inlineStr"/>
+      <c r="AD47" t="inlineStr"/>
+      <c r="AE47" t="inlineStr"/>
+      <c r="AF47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -5176,51 +4524,23 @@
           <t>at/above 200DMA; moving toward 200DMA; above breakdown low; volume &gt;=1.2x</t>
         </is>
       </c>
-      <c r="P48" t="n">
-        <v>143.77863</v>
-      </c>
-      <c r="Q48" t="n">
-        <v>5.813523</v>
-      </c>
-      <c r="R48" t="n">
-        <v>50.23</v>
-      </c>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr"/>
-      <c r="T48" t="n">
-        <v>254703812608</v>
-      </c>
-      <c r="U48" t="n">
-        <v>5.583</v>
-      </c>
+      <c r="T48" t="inlineStr"/>
+      <c r="U48" t="inlineStr"/>
       <c r="V48" t="inlineStr"/>
-      <c r="W48" t="n">
-        <v>6.243</v>
-      </c>
-      <c r="X48" t="n">
-        <v>1.4579999</v>
-      </c>
-      <c r="Y48" t="n">
-        <v>46.566</v>
-      </c>
-      <c r="Z48" t="n">
-        <v>1.131</v>
-      </c>
-      <c r="AA48" t="n">
-        <v>0.476</v>
-      </c>
+      <c r="W48" t="inlineStr"/>
+      <c r="X48" t="inlineStr"/>
+      <c r="Y48" t="inlineStr"/>
+      <c r="Z48" t="inlineStr"/>
+      <c r="AA48" t="inlineStr"/>
       <c r="AB48" t="inlineStr"/>
-      <c r="AC48" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="AD48" t="n">
-        <v>11</v>
-      </c>
-      <c r="AE48" t="n">
-        <v>11</v>
-      </c>
-      <c r="AF48" t="n">
-        <v>33</v>
-      </c>
+      <c r="AC48" t="inlineStr"/>
+      <c r="AD48" t="inlineStr"/>
+      <c r="AE48" t="inlineStr"/>
+      <c r="AF48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -5278,47 +4598,23 @@
           <t>at/above 200DMA; moving toward 200DMA; above breakdown low; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P49" t="n">
-        <v>57.470177</v>
-      </c>
-      <c r="Q49" t="n">
-        <v>8.454114000000001</v>
-      </c>
-      <c r="R49" t="n">
-        <v>57</v>
-      </c>
-      <c r="S49" t="n">
-        <v>8</v>
-      </c>
-      <c r="T49" t="n">
-        <v>246401531904</v>
-      </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr"/>
       <c r="V49" t="inlineStr"/>
-      <c r="W49" t="n">
-        <v>15.506</v>
-      </c>
-      <c r="X49" t="n">
-        <v>11.8389994</v>
-      </c>
-      <c r="Y49" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="W49" t="inlineStr"/>
+      <c r="X49" t="inlineStr"/>
+      <c r="Y49" t="inlineStr"/>
       <c r="Z49" t="inlineStr"/>
       <c r="AA49" t="inlineStr"/>
       <c r="AB49" t="inlineStr"/>
-      <c r="AC49" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="AD49" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="AE49" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="AF49" t="n">
-        <v>62</v>
-      </c>
+      <c r="AC49" t="inlineStr"/>
+      <c r="AD49" t="inlineStr"/>
+      <c r="AE49" t="inlineStr"/>
+      <c r="AF49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -5376,47 +4672,23 @@
           <t>at/above 200DMA; moving toward 200DMA; recovery &gt;=5%</t>
         </is>
       </c>
-      <c r="P50" t="n">
-        <v>67.02742000000001</v>
-      </c>
-      <c r="Q50" t="n">
-        <v>7.0875993</v>
-      </c>
-      <c r="R50" t="n">
-        <v>13.86</v>
-      </c>
-      <c r="S50" t="n">
-        <v>11</v>
-      </c>
-      <c r="T50" t="n">
-        <v>701356113920</v>
-      </c>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
+      <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr"/>
-      <c r="W50" t="n">
-        <v>16.316</v>
-      </c>
-      <c r="X50" t="n">
-        <v>11.023</v>
-      </c>
-      <c r="Y50" t="n">
-        <v>34.15</v>
-      </c>
+      <c r="W50" t="inlineStr"/>
+      <c r="X50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr"/>
       <c r="Z50" t="inlineStr"/>
       <c r="AA50" t="inlineStr"/>
       <c r="AB50" t="inlineStr"/>
-      <c r="AC50" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="AD50" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="AE50" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="AF50" t="n">
-        <v>36</v>
-      </c>
+      <c r="AC50" t="inlineStr"/>
+      <c r="AD50" t="inlineStr"/>
+      <c r="AE50" t="inlineStr"/>
+      <c r="AF50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -5474,43 +4746,23 @@
           <t>at/above 200DMA; moving toward 200DMA; recovery &gt;=5%</t>
         </is>
       </c>
-      <c r="P51" t="n">
-        <v>253.77501</v>
-      </c>
-      <c r="Q51" t="n">
-        <v>-42.687134</v>
-      </c>
-      <c r="R51" t="n">
-        <v>0.4</v>
-      </c>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr"/>
       <c r="S51" t="inlineStr"/>
-      <c r="T51" t="n">
-        <v>1071841673216</v>
-      </c>
+      <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr"/>
-      <c r="W51" t="n">
-        <v>26.193002</v>
-      </c>
-      <c r="X51" t="n">
-        <v>1.1849999</v>
-      </c>
+      <c r="W51" t="inlineStr"/>
+      <c r="X51" t="inlineStr"/>
       <c r="Y51" t="inlineStr"/>
-      <c r="Z51" t="n">
-        <v>0.771</v>
-      </c>
-      <c r="AA51" t="n">
-        <v>0.463</v>
-      </c>
+      <c r="Z51" t="inlineStr"/>
+      <c r="AA51" t="inlineStr"/>
       <c r="AB51" t="inlineStr"/>
-      <c r="AC51" t="n">
-        <v>37.5</v>
-      </c>
+      <c r="AC51" t="inlineStr"/>
       <c r="AD51" t="inlineStr"/>
       <c r="AE51" t="inlineStr"/>
-      <c r="AF51" t="n">
-        <v>35</v>
-      </c>
+      <c r="AF51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -5568,47 +4820,23 @@
           <t>at/above 200DMA; moving toward 200DMA; recovery &gt;=5%</t>
         </is>
       </c>
-      <c r="P52" t="n">
-        <v>38.910156</v>
-      </c>
-      <c r="Q52" t="n">
-        <v>14.310254</v>
-      </c>
-      <c r="R52" t="n">
-        <v>19.59</v>
-      </c>
-      <c r="S52" t="n">
-        <v>166</v>
-      </c>
-      <c r="T52" t="n">
-        <v>189264805888</v>
-      </c>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr"/>
       <c r="U52" t="inlineStr"/>
       <c r="V52" t="inlineStr"/>
-      <c r="W52" t="n">
-        <v>40.046</v>
-      </c>
-      <c r="X52" t="n">
-        <v>31.785</v>
-      </c>
-      <c r="Y52" t="n">
-        <v>4.863</v>
-      </c>
+      <c r="W52" t="inlineStr"/>
+      <c r="X52" t="inlineStr"/>
+      <c r="Y52" t="inlineStr"/>
       <c r="Z52" t="inlineStr"/>
       <c r="AA52" t="inlineStr"/>
       <c r="AB52" t="inlineStr"/>
-      <c r="AC52" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="AD52" t="n">
-        <v>17</v>
-      </c>
-      <c r="AE52" t="n">
-        <v>17</v>
-      </c>
-      <c r="AF52" t="n">
-        <v>56</v>
-      </c>
+      <c r="AC52" t="inlineStr"/>
+      <c r="AD52" t="inlineStr"/>
+      <c r="AE52" t="inlineStr"/>
+      <c r="AF52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -5666,47 +4894,23 @@
           <t>at/above 200DMA; moving toward 200DMA; recovery &gt;=5%</t>
         </is>
       </c>
-      <c r="P53" t="n">
-        <v>29.214525</v>
-      </c>
-      <c r="Q53" t="n">
-        <v>10.045888</v>
-      </c>
-      <c r="R53" t="n">
-        <v>11.84</v>
-      </c>
-      <c r="S53" t="n">
-        <v>145</v>
-      </c>
-      <c r="T53" t="n">
-        <v>149484027904</v>
-      </c>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
+      <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr"/>
-      <c r="W53" t="n">
-        <v>56.596</v>
-      </c>
-      <c r="X53" t="n">
-        <v>44.739</v>
-      </c>
-      <c r="Y53" t="n">
-        <v>9.593999999999999</v>
-      </c>
+      <c r="W53" t="inlineStr"/>
+      <c r="X53" t="inlineStr"/>
+      <c r="Y53" t="inlineStr"/>
       <c r="Z53" t="inlineStr"/>
       <c r="AA53" t="inlineStr"/>
       <c r="AB53" t="inlineStr"/>
-      <c r="AC53" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="AD53" t="n">
-        <v>32</v>
-      </c>
-      <c r="AE53" t="n">
-        <v>32</v>
-      </c>
-      <c r="AF53" t="n">
-        <v>74</v>
-      </c>
+      <c r="AC53" t="inlineStr"/>
+      <c r="AD53" t="inlineStr"/>
+      <c r="AE53" t="inlineStr"/>
+      <c r="AF53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -5764,45 +4968,23 @@
           <t>within 3% of 200DMA; recovery &gt;=5%; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P54" t="n">
-        <v>19.174019</v>
-      </c>
-      <c r="Q54" t="n">
-        <v>2.1468048</v>
-      </c>
-      <c r="R54" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="S54" t="n">
-        <v>17</v>
-      </c>
-      <c r="T54" t="n">
-        <v>3890559844352</v>
-      </c>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr"/>
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr"/>
-      <c r="W54" t="n">
-        <v>34.761003</v>
-      </c>
-      <c r="X54" t="n">
-        <v>28.467</v>
-      </c>
+      <c r="W54" t="inlineStr"/>
+      <c r="X54" t="inlineStr"/>
       <c r="Y54" t="inlineStr"/>
       <c r="Z54" t="inlineStr"/>
       <c r="AA54" t="inlineStr"/>
       <c r="AB54" t="inlineStr"/>
-      <c r="AC54" t="n">
-        <v>21</v>
-      </c>
-      <c r="AD54" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="AE54" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="AF54" t="n">
-        <v>100</v>
-      </c>
+      <c r="AC54" t="inlineStr"/>
+      <c r="AD54" t="inlineStr"/>
+      <c r="AE54" t="inlineStr"/>
+      <c r="AF54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -5860,47 +5042,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; above breakdown low; above 50DMA</t>
         </is>
       </c>
-      <c r="P55" t="n">
-        <v>40.022736</v>
-      </c>
-      <c r="Q55" t="n">
-        <v>4.460094</v>
-      </c>
-      <c r="R55" t="n">
-        <v>290.31</v>
-      </c>
-      <c r="S55" t="n">
-        <v>205</v>
-      </c>
-      <c r="T55" t="n">
-        <v>3417956941824</v>
-      </c>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr"/>
       <c r="U55" t="inlineStr"/>
       <c r="V55" t="inlineStr"/>
-      <c r="W55" t="n">
-        <v>15.478</v>
-      </c>
-      <c r="X55" t="n">
-        <v>9.2930004</v>
-      </c>
-      <c r="Y55" t="n">
-        <v>29.432</v>
-      </c>
+      <c r="W55" t="inlineStr"/>
+      <c r="X55" t="inlineStr"/>
+      <c r="Y55" t="inlineStr"/>
       <c r="Z55" t="inlineStr"/>
       <c r="AA55" t="inlineStr"/>
       <c r="AB55" t="inlineStr"/>
-      <c r="AC55" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="AD55" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="AE55" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="AF55" t="n">
-        <v>44</v>
-      </c>
+      <c r="AC55" t="inlineStr"/>
+      <c r="AD55" t="inlineStr"/>
+      <c r="AE55" t="inlineStr"/>
+      <c r="AF55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -5958,47 +5116,23 @@
           <t>at/above 200DMA; above breakdown low; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P56" t="n">
-        <v>33.773373</v>
-      </c>
-      <c r="Q56" t="n">
-        <v>4.9136887</v>
-      </c>
-      <c r="R56" t="n">
-        <v>62.04</v>
-      </c>
-      <c r="S56" t="n">
-        <v>53</v>
-      </c>
-      <c r="T56" t="n">
-        <v>617058795520</v>
-      </c>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr"/>
       <c r="U56" t="inlineStr"/>
       <c r="V56" t="inlineStr"/>
-      <c r="W56" t="n">
-        <v>6.771999600000001</v>
-      </c>
-      <c r="X56" t="n">
-        <v>5.619</v>
-      </c>
-      <c r="Y56" t="n">
-        <v>11.469</v>
-      </c>
+      <c r="W56" t="inlineStr"/>
+      <c r="X56" t="inlineStr"/>
+      <c r="Y56" t="inlineStr"/>
       <c r="Z56" t="inlineStr"/>
       <c r="AA56" t="inlineStr"/>
       <c r="AB56" t="inlineStr"/>
-      <c r="AC56" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="AD56" t="n">
-        <v>-24.5</v>
-      </c>
-      <c r="AE56" t="n">
-        <v>-24.5</v>
-      </c>
-      <c r="AF56" t="n">
-        <v>30</v>
-      </c>
+      <c r="AC56" t="inlineStr"/>
+      <c r="AD56" t="inlineStr"/>
+      <c r="AE56" t="inlineStr"/>
+      <c r="AF56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -6056,53 +5190,23 @@
           <t>at/above 200DMA; recovery &gt;=5%; above 50DMA</t>
         </is>
       </c>
-      <c r="P57" t="n">
-        <v>17.394787</v>
-      </c>
-      <c r="Q57" t="n">
-        <v>9.694862000000001</v>
-      </c>
-      <c r="R57" t="n">
-        <v>10.74</v>
-      </c>
-      <c r="S57" t="n">
-        <v>667</v>
-      </c>
-      <c r="T57" t="n">
-        <v>184787845120</v>
-      </c>
-      <c r="U57" t="n">
-        <v>56.996</v>
-      </c>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr"/>
+      <c r="U57" t="inlineStr"/>
       <c r="V57" t="inlineStr"/>
-      <c r="W57" t="n">
-        <v>24.779</v>
-      </c>
-      <c r="X57" t="n">
-        <v>17.066</v>
-      </c>
-      <c r="Y57" t="n">
-        <v>2.784</v>
-      </c>
-      <c r="Z57" t="n">
-        <v>1.511</v>
-      </c>
-      <c r="AA57" t="n">
-        <v>0.852</v>
-      </c>
+      <c r="W57" t="inlineStr"/>
+      <c r="X57" t="inlineStr"/>
+      <c r="Y57" t="inlineStr"/>
+      <c r="Z57" t="inlineStr"/>
+      <c r="AA57" t="inlineStr"/>
       <c r="AB57" t="inlineStr"/>
-      <c r="AC57" t="n">
-        <v>25</v>
-      </c>
-      <c r="AD57" t="n">
-        <v>42.1</v>
-      </c>
-      <c r="AE57" t="n">
-        <v>42.1</v>
-      </c>
-      <c r="AF57" t="n">
-        <v>79</v>
-      </c>
+      <c r="AC57" t="inlineStr"/>
+      <c r="AD57" t="inlineStr"/>
+      <c r="AE57" t="inlineStr"/>
+      <c r="AF57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -6160,47 +5264,23 @@
           <t>at/above 200DMA; above breakdown low; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P58" t="n">
-        <v>15.7235565</v>
-      </c>
-      <c r="Q58" t="n">
-        <v>1.7499615</v>
-      </c>
-      <c r="R58" t="n">
-        <v>72.42</v>
-      </c>
-      <c r="S58" t="n">
-        <v>322</v>
-      </c>
-      <c r="T58" t="n">
-        <v>112478248960</v>
-      </c>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr"/>
       <c r="U58" t="inlineStr"/>
       <c r="V58" t="inlineStr"/>
-      <c r="W58" t="n">
-        <v>9.854999000000001</v>
-      </c>
-      <c r="X58" t="n">
-        <v>8.382000000000001</v>
-      </c>
-      <c r="Y58" t="n">
-        <v>3.461</v>
-      </c>
+      <c r="W58" t="inlineStr"/>
+      <c r="X58" t="inlineStr"/>
+      <c r="Y58" t="inlineStr"/>
       <c r="Z58" t="inlineStr"/>
       <c r="AA58" t="inlineStr"/>
       <c r="AB58" t="inlineStr"/>
-      <c r="AC58" t="n">
-        <v>13.9</v>
-      </c>
-      <c r="AD58" t="n">
-        <v>-39.3</v>
-      </c>
-      <c r="AE58" t="n">
-        <v>-39.3</v>
-      </c>
-      <c r="AF58" t="n">
-        <v>42</v>
-      </c>
+      <c r="AC58" t="inlineStr"/>
+      <c r="AD58" t="inlineStr"/>
+      <c r="AE58" t="inlineStr"/>
+      <c r="AF58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -6258,47 +5338,23 @@
           <t>at/above 200DMA; above breakdown low; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P59" t="n">
-        <v>45.71522</v>
-      </c>
-      <c r="Q59" t="n">
-        <v>11.137925</v>
-      </c>
-      <c r="R59" t="n">
-        <v>122.06</v>
-      </c>
-      <c r="S59" t="n">
-        <v>65</v>
-      </c>
-      <c r="T59" t="n">
-        <v>871769178112</v>
-      </c>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr"/>
+      <c r="T59" t="inlineStr"/>
       <c r="U59" t="inlineStr"/>
       <c r="V59" t="inlineStr"/>
-      <c r="W59" t="n">
-        <v>13.516</v>
-      </c>
-      <c r="X59" t="n">
-        <v>12.236</v>
-      </c>
-      <c r="Y59" t="n">
-        <v>6.092</v>
-      </c>
+      <c r="W59" t="inlineStr"/>
+      <c r="X59" t="inlineStr"/>
+      <c r="Y59" t="inlineStr"/>
       <c r="Z59" t="inlineStr"/>
       <c r="AA59" t="inlineStr"/>
       <c r="AB59" t="inlineStr"/>
-      <c r="AC59" t="n">
-        <v>29.1</v>
-      </c>
-      <c r="AD59" t="n">
-        <v>12.1</v>
-      </c>
-      <c r="AE59" t="n">
-        <v>12.1</v>
-      </c>
-      <c r="AF59" t="n">
-        <v>56</v>
-      </c>
+      <c r="AC59" t="inlineStr"/>
+      <c r="AD59" t="inlineStr"/>
+      <c r="AE59" t="inlineStr"/>
+      <c r="AF59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -6357,42 +5413,22 @@
         </is>
       </c>
       <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="n">
-        <v>0.6559713</v>
-      </c>
-      <c r="R60" t="n">
-        <v>-89.77</v>
-      </c>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr"/>
-      <c r="T60" t="n">
-        <v>175048392704</v>
-      </c>
+      <c r="T60" t="inlineStr"/>
       <c r="U60" t="inlineStr"/>
       <c r="V60" t="inlineStr"/>
-      <c r="W60" t="n">
-        <v>93.80199999999999</v>
-      </c>
-      <c r="X60" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y60" t="n">
-        <v>273.033</v>
-      </c>
+      <c r="W60" t="inlineStr"/>
+      <c r="X60" t="inlineStr"/>
+      <c r="Y60" t="inlineStr"/>
       <c r="Z60" t="inlineStr"/>
       <c r="AA60" t="inlineStr"/>
       <c r="AB60" t="inlineStr"/>
-      <c r="AC60" t="n">
-        <v>-52.90000000000001</v>
-      </c>
-      <c r="AD60" t="n">
-        <v>-50</v>
-      </c>
-      <c r="AE60" t="n">
-        <v>-50</v>
-      </c>
-      <c r="AF60" t="n">
-        <v>0</v>
-      </c>
+      <c r="AC60" t="inlineStr"/>
+      <c r="AD60" t="inlineStr"/>
+      <c r="AE60" t="inlineStr"/>
+      <c r="AF60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -6450,47 +5486,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; above breakdown low; volume &gt;=1.2x</t>
         </is>
       </c>
-      <c r="P61" t="n">
-        <v>34.616726</v>
-      </c>
-      <c r="Q61" t="n">
-        <v>5.778402</v>
-      </c>
-      <c r="R61" t="n">
-        <v>8.609999999999999</v>
-      </c>
-      <c r="S61" t="n">
-        <v>6</v>
-      </c>
-      <c r="T61" t="n">
-        <v>89464422400</v>
-      </c>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
+      <c r="T61" t="inlineStr"/>
       <c r="U61" t="inlineStr"/>
       <c r="V61" t="inlineStr"/>
-      <c r="W61" t="n">
-        <v>15.117</v>
-      </c>
-      <c r="X61" t="n">
-        <v>10.132</v>
-      </c>
-      <c r="Y61" t="n">
-        <v>29.595</v>
-      </c>
+      <c r="W61" t="inlineStr"/>
+      <c r="X61" t="inlineStr"/>
+      <c r="Y61" t="inlineStr"/>
       <c r="Z61" t="inlineStr"/>
       <c r="AA61" t="inlineStr"/>
       <c r="AB61" t="inlineStr"/>
-      <c r="AC61" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="AD61" t="n">
-        <v>-8.5</v>
-      </c>
-      <c r="AE61" t="n">
-        <v>-8.5</v>
-      </c>
-      <c r="AF61" t="n">
-        <v>30</v>
-      </c>
+      <c r="AC61" t="inlineStr"/>
+      <c r="AD61" t="inlineStr"/>
+      <c r="AE61" t="inlineStr"/>
+      <c r="AF61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -6548,47 +5560,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; recovery &gt;=5%</t>
         </is>
       </c>
-      <c r="P62" t="n">
-        <v>8.708930000000001</v>
-      </c>
-      <c r="Q62" t="n">
-        <v>2.9618435</v>
-      </c>
-      <c r="R62" t="n">
-        <v>47.48</v>
-      </c>
-      <c r="S62" t="n">
-        <v>243</v>
-      </c>
-      <c r="T62" t="n">
-        <v>2615386570752</v>
-      </c>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
+      <c r="T62" t="inlineStr"/>
       <c r="U62" t="inlineStr"/>
       <c r="V62" t="inlineStr"/>
-      <c r="W62" t="n">
-        <v>6.426</v>
-      </c>
-      <c r="X62" t="n">
-        <v>6.515</v>
-      </c>
-      <c r="Y62" t="n">
-        <v>0.431</v>
-      </c>
+      <c r="W62" t="inlineStr"/>
+      <c r="X62" t="inlineStr"/>
+      <c r="Y62" t="inlineStr"/>
       <c r="Z62" t="inlineStr"/>
       <c r="AA62" t="inlineStr"/>
       <c r="AB62" t="inlineStr"/>
-      <c r="AC62" t="n">
-        <v>6.800000000000001</v>
-      </c>
-      <c r="AD62" t="n">
-        <v>40</v>
-      </c>
-      <c r="AE62" t="n">
-        <v>40</v>
-      </c>
-      <c r="AF62" t="n">
-        <v>76</v>
-      </c>
+      <c r="AC62" t="inlineStr"/>
+      <c r="AD62" t="inlineStr"/>
+      <c r="AE62" t="inlineStr"/>
+      <c r="AF62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -6646,45 +5634,23 @@
           <t>at/above 200DMA; moving toward 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P63" t="n">
-        <v>16.611982</v>
-      </c>
-      <c r="Q63" t="n">
-        <v>2.1909964</v>
-      </c>
-      <c r="R63" t="n">
-        <v>84.12</v>
-      </c>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr"/>
       <c r="S63" t="inlineStr"/>
-      <c r="T63" t="n">
-        <v>110799880192</v>
-      </c>
+      <c r="T63" t="inlineStr"/>
       <c r="U63" t="inlineStr"/>
       <c r="V63" t="inlineStr"/>
-      <c r="W63" t="n">
-        <v>54.527</v>
-      </c>
-      <c r="X63" t="n">
-        <v>42.543998</v>
-      </c>
-      <c r="Y63" t="n">
-        <v>310.553</v>
-      </c>
+      <c r="W63" t="inlineStr"/>
+      <c r="X63" t="inlineStr"/>
+      <c r="Y63" t="inlineStr"/>
       <c r="Z63" t="inlineStr"/>
       <c r="AA63" t="inlineStr"/>
       <c r="AB63" t="inlineStr"/>
-      <c r="AC63" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="AD63" t="n">
-        <v>23.3</v>
-      </c>
-      <c r="AE63" t="n">
-        <v>23.3</v>
-      </c>
-      <c r="AF63" t="n">
-        <v>74</v>
-      </c>
+      <c r="AC63" t="inlineStr"/>
+      <c r="AD63" t="inlineStr"/>
+      <c r="AE63" t="inlineStr"/>
+      <c r="AF63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -6742,47 +5708,23 @@
           <t>at/above 200DMA; moving toward 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P64" t="n">
-        <v>53.19195</v>
-      </c>
-      <c r="Q64" t="n">
-        <v>14.205161</v>
-      </c>
-      <c r="R64" t="n">
-        <v>32.3</v>
-      </c>
-      <c r="S64" t="n">
-        <v>100</v>
-      </c>
-      <c r="T64" t="n">
-        <v>489687252992</v>
-      </c>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr"/>
+      <c r="T64" t="inlineStr"/>
       <c r="U64" t="inlineStr"/>
       <c r="V64" t="inlineStr"/>
-      <c r="W64" t="n">
-        <v>7.454</v>
-      </c>
-      <c r="X64" t="n">
-        <v>3.72</v>
-      </c>
-      <c r="Y64" t="n">
-        <v>335.854</v>
-      </c>
+      <c r="W64" t="inlineStr"/>
+      <c r="X64" t="inlineStr"/>
+      <c r="Y64" t="inlineStr"/>
       <c r="Z64" t="inlineStr"/>
       <c r="AA64" t="inlineStr"/>
       <c r="AB64" t="inlineStr"/>
-      <c r="AC64" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="AD64" t="n">
-        <v>-29.4</v>
-      </c>
-      <c r="AE64" t="n">
-        <v>-29.4</v>
-      </c>
-      <c r="AF64" t="n">
-        <v>22</v>
-      </c>
+      <c r="AC64" t="inlineStr"/>
+      <c r="AD64" t="inlineStr"/>
+      <c r="AE64" t="inlineStr"/>
+      <c r="AF64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -6840,47 +5782,23 @@
           <t>at/above 200DMA; moving toward 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P65" t="n">
-        <v>18.656094</v>
-      </c>
-      <c r="Q65" t="n">
-        <v>4.5517774</v>
-      </c>
-      <c r="R65" t="n">
-        <v>119.8</v>
-      </c>
-      <c r="S65" t="n">
-        <v>80</v>
-      </c>
-      <c r="T65" t="n">
-        <v>1021919952896</v>
-      </c>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr"/>
+      <c r="T65" t="inlineStr"/>
       <c r="U65" t="inlineStr"/>
       <c r="V65" t="inlineStr"/>
-      <c r="W65" t="n">
-        <v>25.354</v>
-      </c>
-      <c r="X65" t="n">
-        <v>18.450001</v>
-      </c>
-      <c r="Y65" t="n">
-        <v>29.388</v>
-      </c>
+      <c r="W65" t="inlineStr"/>
+      <c r="X65" t="inlineStr"/>
+      <c r="Y65" t="inlineStr"/>
       <c r="Z65" t="inlineStr"/>
       <c r="AA65" t="inlineStr"/>
       <c r="AB65" t="inlineStr"/>
-      <c r="AC65" t="n">
-        <v>32</v>
-      </c>
-      <c r="AD65" t="n">
-        <v>16</v>
-      </c>
-      <c r="AE65" t="n">
-        <v>16</v>
-      </c>
-      <c r="AF65" t="n">
-        <v>68</v>
-      </c>
+      <c r="AC65" t="inlineStr"/>
+      <c r="AD65" t="inlineStr"/>
+      <c r="AE65" t="inlineStr"/>
+      <c r="AF65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -6938,45 +5856,23 @@
           <t>at/above 200DMA; moving toward 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P66" t="n">
-        <v>25.202898</v>
-      </c>
-      <c r="Q66" t="n">
-        <v>1.3351247</v>
-      </c>
-      <c r="R66" t="n">
-        <v>0.6899999999999999</v>
-      </c>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr"/>
       <c r="S66" t="inlineStr"/>
-      <c r="T66" t="n">
-        <v>119181647872</v>
-      </c>
+      <c r="T66" t="inlineStr"/>
       <c r="U66" t="inlineStr"/>
       <c r="V66" t="inlineStr"/>
-      <c r="W66" t="n">
-        <v>36.141</v>
-      </c>
-      <c r="X66" t="n">
-        <v>11.1420006</v>
-      </c>
-      <c r="Y66" t="n">
-        <v>26.634</v>
-      </c>
+      <c r="W66" t="inlineStr"/>
+      <c r="X66" t="inlineStr"/>
+      <c r="Y66" t="inlineStr"/>
       <c r="Z66" t="inlineStr"/>
       <c r="AA66" t="inlineStr"/>
       <c r="AB66" t="inlineStr"/>
-      <c r="AC66" t="n">
-        <v>12.2</v>
-      </c>
-      <c r="AD66" t="n">
-        <v>67.7</v>
-      </c>
-      <c r="AE66" t="n">
-        <v>67.7</v>
-      </c>
-      <c r="AF66" t="n">
-        <v>62</v>
-      </c>
+      <c r="AC66" t="inlineStr"/>
+      <c r="AD66" t="inlineStr"/>
+      <c r="AE66" t="inlineStr"/>
+      <c r="AF66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -7034,47 +5930,23 @@
           <t>at/above 200DMA; moving toward 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P67" t="n">
-        <v>66.697</v>
-      </c>
-      <c r="Q67" t="n">
-        <v>12.903393</v>
-      </c>
-      <c r="R67" t="n">
-        <v>9.34</v>
-      </c>
-      <c r="S67" t="n">
-        <v>13</v>
-      </c>
-      <c r="T67" t="n">
-        <v>147324108800</v>
-      </c>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr"/>
+      <c r="T67" t="inlineStr"/>
       <c r="U67" t="inlineStr"/>
       <c r="V67" t="inlineStr"/>
-      <c r="W67" t="n">
-        <v>8.273999999999999</v>
-      </c>
-      <c r="X67" t="n">
-        <v>3.571</v>
-      </c>
-      <c r="Y67" t="n">
-        <v>190.282</v>
-      </c>
+      <c r="W67" t="inlineStr"/>
+      <c r="X67" t="inlineStr"/>
+      <c r="Y67" t="inlineStr"/>
       <c r="Z67" t="inlineStr"/>
       <c r="AA67" t="inlineStr"/>
       <c r="AB67" t="inlineStr"/>
-      <c r="AC67" t="n">
-        <v>15</v>
-      </c>
-      <c r="AD67" t="n">
-        <v>14.1</v>
-      </c>
-      <c r="AE67" t="n">
-        <v>14.1</v>
-      </c>
-      <c r="AF67" t="n">
-        <v>36</v>
-      </c>
+      <c r="AC67" t="inlineStr"/>
+      <c r="AD67" t="inlineStr"/>
+      <c r="AE67" t="inlineStr"/>
+      <c r="AF67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -7132,45 +6004,23 @@
           <t>at/above 200DMA; recovery &gt;=5%; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P68" t="n">
-        <v>21.521738</v>
-      </c>
-      <c r="Q68" t="n">
-        <v>4.552851</v>
-      </c>
-      <c r="R68" t="n">
-        <v>2.99</v>
-      </c>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr"/>
       <c r="S68" t="inlineStr"/>
-      <c r="T68" t="n">
-        <v>96525000704</v>
-      </c>
+      <c r="T68" t="inlineStr"/>
       <c r="U68" t="inlineStr"/>
       <c r="V68" t="inlineStr"/>
-      <c r="W68" t="n">
-        <v>85.238</v>
-      </c>
-      <c r="X68" t="n">
-        <v>573.759</v>
-      </c>
-      <c r="Y68" t="n">
-        <v>0.114</v>
-      </c>
+      <c r="W68" t="inlineStr"/>
+      <c r="X68" t="inlineStr"/>
+      <c r="Y68" t="inlineStr"/>
       <c r="Z68" t="inlineStr"/>
       <c r="AA68" t="inlineStr"/>
       <c r="AB68" t="inlineStr"/>
-      <c r="AC68" t="n">
-        <v>10644.1</v>
-      </c>
-      <c r="AD68" t="n">
-        <v>130</v>
-      </c>
-      <c r="AE68" t="n">
-        <v>130</v>
-      </c>
-      <c r="AF68" t="n">
-        <v>94</v>
-      </c>
+      <c r="AC68" t="inlineStr"/>
+      <c r="AD68" t="inlineStr"/>
+      <c r="AE68" t="inlineStr"/>
+      <c r="AF68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -7228,47 +6078,23 @@
           <t>at/above 200DMA; recovery &gt;=5%; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P69" t="n">
-        <v>37.451374</v>
-      </c>
-      <c r="Q69" t="n">
-        <v>11.421667</v>
-      </c>
-      <c r="R69" t="n">
-        <v>69.92</v>
-      </c>
-      <c r="S69" t="n">
-        <v>102</v>
-      </c>
-      <c r="T69" t="n">
-        <v>299965874176</v>
-      </c>
+      <c r="P69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr"/>
+      <c r="T69" t="inlineStr"/>
       <c r="U69" t="inlineStr"/>
       <c r="V69" t="inlineStr"/>
-      <c r="W69" t="n">
-        <v>7.48</v>
-      </c>
-      <c r="X69" t="n">
-        <v>10.665</v>
-      </c>
-      <c r="Y69" t="n">
-        <v>1.424</v>
-      </c>
+      <c r="W69" t="inlineStr"/>
+      <c r="X69" t="inlineStr"/>
+      <c r="Y69" t="inlineStr"/>
       <c r="Z69" t="inlineStr"/>
       <c r="AA69" t="inlineStr"/>
       <c r="AB69" t="inlineStr"/>
-      <c r="AC69" t="n">
-        <v>38.5</v>
-      </c>
-      <c r="AD69" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="AE69" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="AF69" t="n">
-        <v>70</v>
-      </c>
+      <c r="AC69" t="inlineStr"/>
+      <c r="AD69" t="inlineStr"/>
+      <c r="AE69" t="inlineStr"/>
+      <c r="AF69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -7326,45 +6152,23 @@
           <t>at/above 200DMA; moving toward 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P70" t="n">
-        <v>19.340063</v>
-      </c>
-      <c r="Q70" t="n">
-        <v>2.8785374</v>
-      </c>
-      <c r="R70" t="n">
-        <v>25.76</v>
-      </c>
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr"/>
       <c r="S70" t="inlineStr"/>
-      <c r="T70" t="n">
-        <v>218080821248</v>
-      </c>
+      <c r="T70" t="inlineStr"/>
       <c r="U70" t="inlineStr"/>
       <c r="V70" t="inlineStr"/>
-      <c r="W70" t="n">
-        <v>61.72299999999999</v>
-      </c>
-      <c r="X70" t="n">
-        <v>48.151</v>
-      </c>
-      <c r="Y70" t="n">
-        <v>255.574</v>
-      </c>
+      <c r="W70" t="inlineStr"/>
+      <c r="X70" t="inlineStr"/>
+      <c r="Y70" t="inlineStr"/>
       <c r="Z70" t="inlineStr"/>
       <c r="AA70" t="inlineStr"/>
       <c r="AB70" t="inlineStr"/>
-      <c r="AC70" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="AD70" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="AE70" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="AF70" t="n">
-        <v>68</v>
-      </c>
+      <c r="AC70" t="inlineStr"/>
+      <c r="AD70" t="inlineStr"/>
+      <c r="AE70" t="inlineStr"/>
+      <c r="AF70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -7422,47 +6226,23 @@
           <t>within 3% of 200DMA; above breakdown low; above 50DMA; RSI &gt;=50</t>
         </is>
       </c>
-      <c r="P71" t="n">
-        <v>40.83427</v>
-      </c>
-      <c r="Q71" t="n">
-        <v>2.1815078</v>
-      </c>
-      <c r="R71" t="n">
-        <v>26.73</v>
-      </c>
-      <c r="S71" t="n">
-        <v>18</v>
-      </c>
-      <c r="T71" t="n">
-        <v>1110588260352</v>
-      </c>
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr"/>
+      <c r="T71" t="inlineStr"/>
       <c r="U71" t="inlineStr"/>
       <c r="V71" t="inlineStr"/>
-      <c r="W71" t="n">
-        <v>11.1999996</v>
-      </c>
-      <c r="X71" t="n">
-        <v>4.818</v>
-      </c>
-      <c r="Y71" t="n">
-        <v>43.613</v>
-      </c>
+      <c r="W71" t="inlineStr"/>
+      <c r="X71" t="inlineStr"/>
+      <c r="Y71" t="inlineStr"/>
       <c r="Z71" t="inlineStr"/>
       <c r="AA71" t="inlineStr"/>
       <c r="AB71" t="inlineStr"/>
-      <c r="AC71" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="AD71" t="n">
-        <v>-43.7</v>
-      </c>
-      <c r="AE71" t="n">
-        <v>-43.7</v>
-      </c>
-      <c r="AF71" t="n">
-        <v>36</v>
-      </c>
+      <c r="AC71" t="inlineStr"/>
+      <c r="AD71" t="inlineStr"/>
+      <c r="AE71" t="inlineStr"/>
+      <c r="AF71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -7520,53 +6300,23 @@
           <t>at/above 200DMA; recovery &gt;=10%</t>
         </is>
       </c>
-      <c r="P72" t="n">
-        <v>10.035672</v>
-      </c>
-      <c r="Q72" t="n">
-        <v>2.1744733</v>
-      </c>
-      <c r="R72" t="n">
-        <v>8.41</v>
-      </c>
-      <c r="S72" t="n">
-        <v>412</v>
-      </c>
-      <c r="T72" t="n">
-        <v>742029393920</v>
-      </c>
-      <c r="U72" t="n">
-        <v>23.363</v>
-      </c>
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr"/>
+      <c r="T72" t="inlineStr"/>
+      <c r="U72" t="inlineStr"/>
       <c r="V72" t="inlineStr"/>
-      <c r="W72" t="n">
-        <v>21.968001</v>
-      </c>
-      <c r="X72" t="n">
-        <v>23.231001</v>
-      </c>
-      <c r="Y72" t="n">
-        <v>18.802</v>
-      </c>
-      <c r="Z72" t="n">
-        <v>2.429</v>
-      </c>
-      <c r="AA72" t="n">
-        <v>1.702</v>
-      </c>
+      <c r="W72" t="inlineStr"/>
+      <c r="X72" t="inlineStr"/>
+      <c r="Y72" t="inlineStr"/>
+      <c r="Z72" t="inlineStr"/>
+      <c r="AA72" t="inlineStr"/>
       <c r="AB72" t="inlineStr"/>
-      <c r="AC72" t="n">
-        <v>61.9</v>
-      </c>
-      <c r="AD72" t="n">
-        <v>37.7</v>
-      </c>
-      <c r="AE72" t="n">
-        <v>37.7</v>
-      </c>
-      <c r="AF72" t="n">
-        <v>86</v>
-      </c>
+      <c r="AC72" t="inlineStr"/>
+      <c r="AD72" t="inlineStr"/>
+      <c r="AE72" t="inlineStr"/>
+      <c r="AF72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -7625,38 +6375,22 @@
         </is>
       </c>
       <c r="P73" t="inlineStr"/>
-      <c r="Q73" t="n">
-        <v>3.0729208</v>
-      </c>
-      <c r="R73" t="n">
-        <v>-4.24</v>
-      </c>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
       <c r="S73" t="inlineStr"/>
-      <c r="T73" t="n">
-        <v>178797969408</v>
-      </c>
+      <c r="T73" t="inlineStr"/>
       <c r="U73" t="inlineStr"/>
       <c r="V73" t="inlineStr"/>
-      <c r="W73" t="n">
-        <v>11.492</v>
-      </c>
-      <c r="X73" t="n">
-        <v>-3.15</v>
-      </c>
-      <c r="Y73" t="n">
-        <v>25.791</v>
-      </c>
+      <c r="W73" t="inlineStr"/>
+      <c r="X73" t="inlineStr"/>
+      <c r="Y73" t="inlineStr"/>
       <c r="Z73" t="inlineStr"/>
       <c r="AA73" t="inlineStr"/>
       <c r="AB73" t="inlineStr"/>
-      <c r="AC73" t="n">
-        <v>37.2</v>
-      </c>
+      <c r="AC73" t="inlineStr"/>
       <c r="AD73" t="inlineStr"/>
       <c r="AE73" t="inlineStr"/>
-      <c r="AF73" t="n">
-        <v>33</v>
-      </c>
+      <c r="AF73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -7714,47 +6448,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P74" t="n">
-        <v>4.903233</v>
-      </c>
-      <c r="Q74" t="n">
-        <v>1.081117</v>
-      </c>
-      <c r="R74" t="n">
-        <v>261.97</v>
-      </c>
-      <c r="S74" t="n">
-        <v>443</v>
-      </c>
-      <c r="T74" t="n">
-        <v>183387652096</v>
-      </c>
+      <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="inlineStr"/>
       <c r="U74" t="inlineStr"/>
       <c r="V74" t="inlineStr"/>
-      <c r="W74" t="n">
-        <v>54.431</v>
-      </c>
-      <c r="X74" t="n">
-        <v>60.307</v>
-      </c>
-      <c r="Y74" t="n">
-        <v>6.409</v>
-      </c>
+      <c r="W74" t="inlineStr"/>
+      <c r="X74" t="inlineStr"/>
+      <c r="Y74" t="inlineStr"/>
       <c r="Z74" t="inlineStr"/>
       <c r="AA74" t="inlineStr"/>
       <c r="AB74" t="inlineStr"/>
-      <c r="AC74" t="n">
-        <v>66.90000000000001</v>
-      </c>
-      <c r="AD74" t="n">
-        <v>159.4</v>
-      </c>
-      <c r="AE74" t="n">
-        <v>159.4</v>
-      </c>
-      <c r="AF74" t="n">
-        <v>80</v>
-      </c>
+      <c r="AC74" t="inlineStr"/>
+      <c r="AD74" t="inlineStr"/>
+      <c r="AE74" t="inlineStr"/>
+      <c r="AF74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -7812,47 +6522,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P75" t="n">
-        <v>11.590909</v>
-      </c>
-      <c r="Q75" t="n">
-        <v>1.7740043</v>
-      </c>
-      <c r="R75" t="n">
-        <v>23.76</v>
-      </c>
-      <c r="S75" t="n">
-        <v>262</v>
-      </c>
-      <c r="T75" t="n">
-        <v>381879746560</v>
-      </c>
+      <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr"/>
+      <c r="T75" t="inlineStr"/>
       <c r="U75" t="inlineStr"/>
       <c r="V75" t="inlineStr"/>
-      <c r="W75" t="n">
-        <v>28.304002</v>
-      </c>
-      <c r="X75" t="n">
-        <v>17.458001</v>
-      </c>
-      <c r="Y75" t="n">
-        <v>82</v>
-      </c>
+      <c r="W75" t="inlineStr"/>
+      <c r="X75" t="inlineStr"/>
+      <c r="Y75" t="inlineStr"/>
       <c r="Z75" t="inlineStr"/>
       <c r="AA75" t="inlineStr"/>
       <c r="AB75" t="inlineStr"/>
-      <c r="AC75" t="n">
-        <v>-0.3</v>
-      </c>
-      <c r="AD75" t="n">
-        <v>-12.7</v>
-      </c>
-      <c r="AE75" t="n">
-        <v>-12.7</v>
-      </c>
-      <c r="AF75" t="n">
-        <v>34</v>
-      </c>
+      <c r="AC75" t="inlineStr"/>
+      <c r="AD75" t="inlineStr"/>
+      <c r="AE75" t="inlineStr"/>
+      <c r="AF75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -7910,47 +6596,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P76" t="n">
-        <v>20.555058</v>
-      </c>
-      <c r="Q76" t="n">
-        <v>2.760321</v>
-      </c>
-      <c r="R76" t="n">
-        <v>33.42</v>
-      </c>
-      <c r="S76" t="n">
-        <v>57.99999999999999</v>
-      </c>
-      <c r="T76" t="n">
-        <v>569106890752</v>
-      </c>
+      <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr"/>
+      <c r="T76" t="inlineStr"/>
       <c r="U76" t="inlineStr"/>
       <c r="V76" t="inlineStr"/>
-      <c r="W76" t="n">
-        <v>42.416</v>
-      </c>
-      <c r="X76" t="n">
-        <v>29.786</v>
-      </c>
-      <c r="Y76" t="n">
-        <v>484.313</v>
-      </c>
+      <c r="W76" t="inlineStr"/>
+      <c r="X76" t="inlineStr"/>
+      <c r="Y76" t="inlineStr"/>
       <c r="Z76" t="inlineStr"/>
       <c r="AA76" t="inlineStr"/>
       <c r="AB76" t="inlineStr"/>
-      <c r="AC76" t="n">
-        <v>21</v>
-      </c>
-      <c r="AD76" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="AE76" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="AF76" t="n">
-        <v>74</v>
-      </c>
+      <c r="AC76" t="inlineStr"/>
+      <c r="AD76" t="inlineStr"/>
+      <c r="AE76" t="inlineStr"/>
+      <c r="AF76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -8008,47 +6670,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P77" t="n">
-        <v>19.721561</v>
-      </c>
-      <c r="Q77" t="n">
-        <v>2.6128383</v>
-      </c>
-      <c r="R77" t="n">
-        <v>29.45</v>
-      </c>
-      <c r="S77" t="n">
-        <v>170</v>
-      </c>
-      <c r="T77" t="n">
-        <v>184694390784</v>
-      </c>
+      <c r="P77" t="inlineStr"/>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr"/>
+      <c r="T77" t="inlineStr"/>
       <c r="U77" t="inlineStr"/>
       <c r="V77" t="inlineStr"/>
-      <c r="W77" t="n">
-        <v>17.395</v>
-      </c>
-      <c r="X77" t="n">
-        <v>33.823</v>
-      </c>
-      <c r="Y77" t="n">
-        <v>4.475</v>
-      </c>
+      <c r="W77" t="inlineStr"/>
+      <c r="X77" t="inlineStr"/>
+      <c r="Y77" t="inlineStr"/>
       <c r="Z77" t="inlineStr"/>
       <c r="AA77" t="inlineStr"/>
       <c r="AB77" t="inlineStr"/>
-      <c r="AC77" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="AD77" t="n">
-        <v>-0.2</v>
-      </c>
-      <c r="AE77" t="n">
-        <v>-0.2</v>
-      </c>
-      <c r="AF77" t="n">
-        <v>60</v>
-      </c>
+      <c r="AC77" t="inlineStr"/>
+      <c r="AD77" t="inlineStr"/>
+      <c r="AE77" t="inlineStr"/>
+      <c r="AF77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -8106,47 +6744,23 @@
           <t>within 3% of 200DMA; moving toward 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P78" t="n">
-        <v>45.249382</v>
-      </c>
-      <c r="Q78" t="n">
-        <v>8.203222999999999</v>
-      </c>
-      <c r="R78" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="S78" t="n">
-        <v>25</v>
-      </c>
-      <c r="T78" t="n">
-        <v>372200767488</v>
-      </c>
+      <c r="P78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr"/>
+      <c r="T78" t="inlineStr"/>
       <c r="U78" t="inlineStr"/>
       <c r="V78" t="inlineStr"/>
-      <c r="W78" t="n">
-        <v>12.839</v>
-      </c>
-      <c r="X78" t="n">
-        <v>8.984</v>
-      </c>
-      <c r="Y78" t="n">
-        <v>129.033</v>
-      </c>
+      <c r="W78" t="inlineStr"/>
+      <c r="X78" t="inlineStr"/>
+      <c r="Y78" t="inlineStr"/>
       <c r="Z78" t="inlineStr"/>
       <c r="AA78" t="inlineStr"/>
       <c r="AB78" t="inlineStr"/>
-      <c r="AC78" t="n">
-        <v>80.40000000000001</v>
-      </c>
-      <c r="AD78" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="AE78" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="AF78" t="n">
-        <v>44</v>
-      </c>
+      <c r="AC78" t="inlineStr"/>
+      <c r="AD78" t="inlineStr"/>
+      <c r="AE78" t="inlineStr"/>
+      <c r="AF78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -8204,53 +6818,23 @@
           <t>within 3% of 200DMA; above breakdown low; volume &gt;=1.2x</t>
         </is>
       </c>
-      <c r="P79" t="n">
-        <v>20.569326</v>
-      </c>
-      <c r="Q79" t="n">
-        <v>1.8531164</v>
-      </c>
-      <c r="R79" t="n">
-        <v>27.84</v>
-      </c>
-      <c r="S79" t="n">
-        <v>144</v>
-      </c>
-      <c r="T79" t="n">
-        <v>162278129664</v>
-      </c>
-      <c r="U79" t="n">
-        <v>10.309</v>
-      </c>
+      <c r="P79" t="inlineStr"/>
+      <c r="Q79" t="inlineStr"/>
+      <c r="R79" t="inlineStr"/>
+      <c r="S79" t="inlineStr"/>
+      <c r="T79" t="inlineStr"/>
+      <c r="U79" t="inlineStr"/>
       <c r="V79" t="inlineStr"/>
-      <c r="W79" t="n">
-        <v>25.088</v>
-      </c>
-      <c r="X79" t="n">
-        <v>18.333</v>
-      </c>
-      <c r="Y79" t="n">
-        <v>20.684</v>
-      </c>
-      <c r="Z79" t="n">
-        <v>7.59</v>
-      </c>
-      <c r="AA79" t="n">
-        <v>6.018</v>
-      </c>
+      <c r="W79" t="inlineStr"/>
+      <c r="X79" t="inlineStr"/>
+      <c r="Y79" t="inlineStr"/>
+      <c r="Z79" t="inlineStr"/>
+      <c r="AA79" t="inlineStr"/>
       <c r="AB79" t="inlineStr"/>
-      <c r="AC79" t="n">
-        <v>12.2</v>
-      </c>
-      <c r="AD79" t="n">
-        <v>-44.6</v>
-      </c>
-      <c r="AE79" t="n">
-        <v>-44.6</v>
-      </c>
-      <c r="AF79" t="n">
-        <v>51</v>
-      </c>
+      <c r="AC79" t="inlineStr"/>
+      <c r="AD79" t="inlineStr"/>
+      <c r="AE79" t="inlineStr"/>
+      <c r="AF79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -8308,47 +6892,23 @@
           <t>within 3% of 200DMA; above breakdown low; volume &gt;=1.2x</t>
         </is>
       </c>
-      <c r="P80" t="n">
-        <v>83.33842</v>
-      </c>
-      <c r="Q80" t="n">
-        <v>6.825559</v>
-      </c>
-      <c r="R80" t="n">
-        <v>32.8</v>
-      </c>
-      <c r="S80" t="n">
-        <v>16</v>
-      </c>
-      <c r="T80" t="n">
-        <v>529129930752</v>
-      </c>
+      <c r="P80" t="inlineStr"/>
+      <c r="Q80" t="inlineStr"/>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="inlineStr"/>
+      <c r="T80" t="inlineStr"/>
       <c r="U80" t="inlineStr"/>
       <c r="V80" t="inlineStr"/>
-      <c r="W80" t="n">
-        <v>7.277</v>
-      </c>
-      <c r="X80" t="n">
-        <v>2.8169999</v>
-      </c>
-      <c r="Y80" t="n">
-        <v>27.724</v>
-      </c>
+      <c r="W80" t="inlineStr"/>
+      <c r="X80" t="inlineStr"/>
+      <c r="Y80" t="inlineStr"/>
       <c r="Z80" t="inlineStr"/>
       <c r="AA80" t="inlineStr"/>
       <c r="AB80" t="inlineStr"/>
-      <c r="AC80" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="AD80" t="n">
-        <v>-14.2</v>
-      </c>
-      <c r="AE80" t="n">
-        <v>-14.2</v>
-      </c>
-      <c r="AF80" t="n">
-        <v>28</v>
-      </c>
+      <c r="AC80" t="inlineStr"/>
+      <c r="AD80" t="inlineStr"/>
+      <c r="AE80" t="inlineStr"/>
+      <c r="AF80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -8406,45 +6966,23 @@
           <t>at/above 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P81" t="n">
-        <v>20.954382</v>
-      </c>
-      <c r="Q81" t="n">
-        <v>1.0980474</v>
-      </c>
-      <c r="R81" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="S81" t="n">
-        <v>85</v>
-      </c>
-      <c r="T81" t="n">
-        <v>281219530752</v>
-      </c>
+      <c r="P81" t="inlineStr"/>
+      <c r="Q81" t="inlineStr"/>
+      <c r="R81" t="inlineStr"/>
+      <c r="S81" t="inlineStr"/>
+      <c r="T81" t="inlineStr"/>
       <c r="U81" t="inlineStr"/>
       <c r="V81" t="inlineStr"/>
-      <c r="W81" t="n">
-        <v>23.771</v>
-      </c>
-      <c r="X81" t="n">
-        <v>13.617</v>
-      </c>
+      <c r="W81" t="inlineStr"/>
+      <c r="X81" t="inlineStr"/>
       <c r="Y81" t="inlineStr"/>
       <c r="Z81" t="inlineStr"/>
       <c r="AA81" t="inlineStr"/>
       <c r="AB81" t="inlineStr"/>
-      <c r="AC81" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="AD81" t="n">
-        <v>34.59999999999999</v>
-      </c>
-      <c r="AE81" t="n">
-        <v>34.59999999999999</v>
-      </c>
-      <c r="AF81" t="n">
-        <v>85</v>
-      </c>
+      <c r="AC81" t="inlineStr"/>
+      <c r="AD81" t="inlineStr"/>
+      <c r="AE81" t="inlineStr"/>
+      <c r="AF81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -8502,45 +7040,23 @@
           <t>at/above 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P82" t="n">
-        <v>14.744877</v>
-      </c>
-      <c r="Q82" t="n">
-        <v>1.9565442</v>
-      </c>
-      <c r="R82" t="n">
-        <v>14.15</v>
-      </c>
-      <c r="S82" t="n">
-        <v>96</v>
-      </c>
-      <c r="T82" t="n">
-        <v>206717861888</v>
-      </c>
+      <c r="P82" t="inlineStr"/>
+      <c r="Q82" t="inlineStr"/>
+      <c r="R82" t="inlineStr"/>
+      <c r="S82" t="inlineStr"/>
+      <c r="T82" t="inlineStr"/>
       <c r="U82" t="inlineStr"/>
       <c r="V82" t="inlineStr"/>
-      <c r="W82" t="n">
-        <v>50.985</v>
-      </c>
-      <c r="X82" t="n">
-        <v>37.791002</v>
-      </c>
+      <c r="W82" t="inlineStr"/>
+      <c r="X82" t="inlineStr"/>
       <c r="Y82" t="inlineStr"/>
       <c r="Z82" t="inlineStr"/>
       <c r="AA82" t="inlineStr"/>
       <c r="AB82" t="inlineStr"/>
-      <c r="AC82" t="n">
-        <v>23.3</v>
-      </c>
-      <c r="AD82" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="AE82" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="AF82" t="n">
-        <v>100</v>
-      </c>
+      <c r="AC82" t="inlineStr"/>
+      <c r="AD82" t="inlineStr"/>
+      <c r="AE82" t="inlineStr"/>
+      <c r="AF82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -8598,47 +7114,23 @@
           <t>within 3% of 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P83" t="n">
-        <v>9.207571</v>
-      </c>
-      <c r="Q83" t="n">
-        <v>1.7019919</v>
-      </c>
-      <c r="R83" t="n">
-        <v>48.08</v>
-      </c>
-      <c r="S83" t="n">
-        <v>271</v>
-      </c>
-      <c r="T83" t="n">
-        <v>177368776704</v>
-      </c>
+      <c r="P83" t="inlineStr"/>
+      <c r="Q83" t="inlineStr"/>
+      <c r="R83" t="inlineStr"/>
+      <c r="S83" t="inlineStr"/>
+      <c r="T83" t="inlineStr"/>
       <c r="U83" t="inlineStr"/>
       <c r="V83" t="inlineStr"/>
-      <c r="W83" t="n">
-        <v>15.151</v>
-      </c>
-      <c r="X83" t="n">
-        <v>9.581000000000001</v>
-      </c>
-      <c r="Y83" t="n">
-        <v>10.274</v>
-      </c>
+      <c r="W83" t="inlineStr"/>
+      <c r="X83" t="inlineStr"/>
+      <c r="Y83" t="inlineStr"/>
       <c r="Z83" t="inlineStr"/>
       <c r="AA83" t="inlineStr"/>
       <c r="AB83" t="inlineStr"/>
-      <c r="AC83" t="n">
-        <v>-11.8</v>
-      </c>
-      <c r="AD83" t="n">
-        <v>-4.6</v>
-      </c>
-      <c r="AE83" t="n">
-        <v>-4.6</v>
-      </c>
-      <c r="AF83" t="n">
-        <v>28</v>
-      </c>
+      <c r="AC83" t="inlineStr"/>
+      <c r="AD83" t="inlineStr"/>
+      <c r="AE83" t="inlineStr"/>
+      <c r="AF83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -8696,47 +7188,23 @@
           <t>within 3% of 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P84" t="n">
-        <v>28.168499</v>
-      </c>
-      <c r="Q84" t="n">
-        <v>1.8688183</v>
-      </c>
-      <c r="R84" t="n">
-        <v>2.73</v>
-      </c>
-      <c r="S84" t="n">
-        <v>209</v>
-      </c>
-      <c r="T84" t="n">
-        <v>772463198208</v>
-      </c>
+      <c r="P84" t="inlineStr"/>
+      <c r="Q84" t="inlineStr"/>
+      <c r="R84" t="inlineStr"/>
+      <c r="S84" t="inlineStr"/>
+      <c r="T84" t="inlineStr"/>
       <c r="U84" t="inlineStr"/>
       <c r="V84" t="inlineStr"/>
-      <c r="W84" t="n">
-        <v>46.019</v>
-      </c>
-      <c r="X84" t="n">
-        <v>31.094998</v>
-      </c>
-      <c r="Y84" t="n">
-        <v>113.111</v>
-      </c>
+      <c r="W84" t="inlineStr"/>
+      <c r="X84" t="inlineStr"/>
+      <c r="Y84" t="inlineStr"/>
       <c r="Z84" t="inlineStr"/>
       <c r="AA84" t="inlineStr"/>
       <c r="AB84" t="inlineStr"/>
-      <c r="AC84" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="AD84" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="AE84" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="AF84" t="n">
-        <v>56</v>
-      </c>
+      <c r="AC84" t="inlineStr"/>
+      <c r="AD84" t="inlineStr"/>
+      <c r="AE84" t="inlineStr"/>
+      <c r="AF84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -8794,47 +7262,23 @@
           <t>within 3% of 200DMA; above breakdown low</t>
         </is>
       </c>
-      <c r="P85" t="n">
-        <v>79.34601600000001</v>
-      </c>
-      <c r="Q85" t="n">
-        <v>1.1554037</v>
-      </c>
-      <c r="R85" t="n">
-        <v>8.41</v>
-      </c>
-      <c r="S85" t="n">
-        <v>50</v>
-      </c>
-      <c r="T85" t="n">
-        <v>337622401024</v>
-      </c>
+      <c r="P85" t="inlineStr"/>
+      <c r="Q85" t="inlineStr"/>
+      <c r="R85" t="inlineStr"/>
+      <c r="S85" t="inlineStr"/>
+      <c r="T85" t="inlineStr"/>
       <c r="U85" t="inlineStr"/>
       <c r="V85" t="inlineStr"/>
-      <c r="W85" t="n">
-        <v>91.65100000000001</v>
-      </c>
-      <c r="X85" t="n">
-        <v>105.248</v>
-      </c>
-      <c r="Y85" t="n">
-        <v>0.007</v>
-      </c>
+      <c r="W85" t="inlineStr"/>
+      <c r="X85" t="inlineStr"/>
+      <c r="Y85" t="inlineStr"/>
       <c r="Z85" t="inlineStr"/>
       <c r="AA85" t="inlineStr"/>
       <c r="AB85" t="inlineStr"/>
-      <c r="AC85" t="n">
-        <v>4.100000000000001</v>
-      </c>
-      <c r="AD85" t="n">
-        <v>-1.8</v>
-      </c>
-      <c r="AE85" t="n">
-        <v>-1.8</v>
-      </c>
-      <c r="AF85" t="n">
-        <v>48</v>
-      </c>
+      <c r="AC85" t="inlineStr"/>
+      <c r="AD85" t="inlineStr"/>
+      <c r="AE85" t="inlineStr"/>
+      <c r="AF85" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>